<commit_message>
Republish with new canonical fhir.heartlandprotocol.org + CNAME
</commit_message>
<xml_diff>
--- a/CodeSystem-heartland-evidence-level.xlsx
+++ b/CodeSystem-heartland-evidence-level.xlsx
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://heartlandprotocol.org/fhir/CodeSystem/heartland-evidence-level</t>
+    <t>https://fhir.heartlandprotocol.org/CodeSystem/heartland-evidence-level</t>
   </si>
   <si>
     <t>Version</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-16T15:03:58-04:00</t>
+    <t>2026-04-16T15:20:02-04:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>